<commit_message>
alteration s post RAG3 iter2_epoch3 final generator+ LLM judge evaluation in ct-pipline
</commit_message>
<xml_diff>
--- a/RAG_CT_complete_compressed/RAG3/iter1_2_macro-metrics.xlsx
+++ b/RAG_CT_complete_compressed/RAG3/iter1_2_macro-metrics.xlsx
@@ -4,19 +4,20 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="36" windowWidth="22980" windowHeight="9552" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="36" windowWidth="22980" windowHeight="9552" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="172">
   <si>
     <r>
       <t>✓</t>
@@ -480,6 +481,102 @@
   </si>
   <si>
     <t>File: /kaggle/working/rag3_evaluation/rag3_complete_evaluation.csv</t>
+  </si>
+  <si>
+    <t>RAG3 o/p(iter2, epoch 3):-</t>
+  </si>
+  <si>
+    <t>RAG3 o/p(iter2, epoch 2):-</t>
+  </si>
+  <si>
+    <t>base_rougeL          0.684971</t>
+  </si>
+  <si>
+    <t>lora_rougeL          0.690823</t>
+  </si>
+  <si>
+    <t>base_bertscore_f1    0.943861</t>
+  </si>
+  <si>
+    <t>lora_bertscore_f1    0.945544</t>
+  </si>
+  <si>
+    <t>Base numeric-grounding issues: 63</t>
+  </si>
+  <si>
+    <t>LoRA numeric-grounding issues: 65</t>
+  </si>
+  <si>
+    <t>base_numeric_groundedness    0.964547</t>
+  </si>
+  <si>
+    <t>lora_numeric_groundedness    0.967221</t>
+  </si>
+  <si>
+    <t>base_numeric_recall          0.891752</t>
+  </si>
+  <si>
+    <t>lora_numeric_recall          0.894615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">             ROUGE-L 0.684971 0.690823    0.005852      0.854281</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        BERTScore-F1 0.943861 0.945544    0.001683      0.178310</t>
+  </si>
+  <si>
+    <t>Numeric groundedness 0.964547 0.967221    0.002674      0.277230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      Numeric recall 0.891752 0.894615    0.002863      0.321032</t>
+  </si>
+  <si>
+    <t>Eligibility / Qualification       228     0.656928     0.657644        0.932666        0.933110         0.910152         0.913755         0.847881         0.836647</t>
+  </si>
+  <si>
+    <t xml:space="preserve">               Intervention        64     0.661598     0.667439        0.943098        0.945551         0.984375         0.996875         0.867188         0.911551</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        Numeric / Threshold        37     0.663168     0.669361        0.939437        0.941543         0.966860         0.966860         0.855143         0.855143</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                      Other       180     0.594660     0.609685        0.934415        0.937659         0.987037         0.990139         0.868108         0.884127</t>
+  </si>
+  <si>
+    <t xml:space="preserve">               Study Design       227     0.809468     0.818702        0.965400        0.967680         0.987885         0.987518         0.964391         0.966960</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                   Temporal        48     0.616053     0.595652        0.935034        0.932568         1.000000         1.000000         0.906250         0.875000</t>
+  </si>
+  <si>
+    <t>Tie     375</t>
+  </si>
+  <si>
+    <t>LoRA    216</t>
+  </si>
+  <si>
+    <t>Base    193</t>
+  </si>
+  <si>
+    <t>LoRA    291</t>
+  </si>
+  <si>
+    <t>Tie     262</t>
+  </si>
+  <si>
+    <t>Base    231</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Mean context-support score 0.443536 0.443660</t>
+  </si>
+  <si>
+    <t>Mean low-support sentence rate 0.018495 0.019770</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Mean numeric groundedness 0.964547 0.967221</t>
+  </si>
+  <si>
+    <t xml:space="preserve">           Mean numeric recall 0.891752 0.894615</t>
   </si>
 </sst>
 </file>
@@ -1659,7 +1756,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18">
       <c r="A1" s="8" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:1">
@@ -2007,5 +2104,360 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A79"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" spans="1:1" ht="18">
+      <c r="A1" s="8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" s="10" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" s="10" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" s="9"/>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" s="10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" s="10" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" s="10" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" s="9"/>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" s="10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" s="10" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" s="10" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" s="10" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" s="10" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" s="10" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" s="10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" s="9"/>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" s="10" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" s="10" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" s="10" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" s="10" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" s="9"/>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" s="10" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" s="10" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" s="9"/>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" s="10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" s="10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" s="10" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" s="10" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" s="10" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" s="10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" s="9"/>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" s="10" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" s="10" t="s">
+        <v>139</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>